<commit_message>
ingesta: snapshot 2026-08-04 18:44 UTC
</commit_message>
<xml_diff>
--- a/data_lake/acumulado_tempmax_mes/dt=2026-08-04/Temp-max-agosto-26.xlsx
+++ b/data_lake/acumulado_tempmax_mes/dt=2026-08-04/Temp-max-agosto-26.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\Mi unidad\OSPA\02. Datos Diarios\Tablas\Datos hidrometeorologicos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\192.168.187.8\Oficina\Mi unidad\OSPA\02. Datos Diarios\Tablas\Datos hidrometeorologicos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00AFF7B9-BA69-44C7-BECB-011956AAD60E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A5C7148-3975-4EA6-8E68-06E3CB942155}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="355" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9419,7 +9419,9 @@
       <c r="F5" s="63">
         <v>31.6</v>
       </c>
-      <c r="G5" s="63"/>
+      <c r="G5" s="63">
+        <v>30.6</v>
+      </c>
       <c r="H5" s="63"/>
       <c r="I5" s="63"/>
       <c r="J5" s="63"/>
@@ -9450,7 +9452,7 @@
       <c r="AI5" s="63"/>
       <c r="AJ5" s="36">
         <f>+IF(SUM($E5:$AI5)&gt;0,LOOKUP(1000,$E5:$AI5),NA())</f>
-        <v>31.6</v>
+        <v>30.6</v>
       </c>
       <c r="AK5" s="21">
         <f>+MAX($E5:$AI5)</f>
@@ -9494,7 +9496,9 @@
       <c r="F6" s="63">
         <v>31</v>
       </c>
-      <c r="G6" s="63"/>
+      <c r="G6" s="63">
+        <v>32.200000000000003</v>
+      </c>
       <c r="H6" s="63"/>
       <c r="I6" s="63"/>
       <c r="J6" s="63"/>
@@ -9525,18 +9529,18 @@
       <c r="AI6" s="63"/>
       <c r="AJ6" s="36">
         <f t="shared" ref="AJ6:AJ48" si="0">+IF(SUM($E6:$AI6)&gt;0,LOOKUP(1000,$E6:$AI6),NA())</f>
-        <v>31</v>
+        <v>32.200000000000003</v>
       </c>
       <c r="AK6" s="21">
         <f t="shared" ref="AK6:AK48" si="1">+MAX($E6:$AI6)</f>
-        <v>31.5</v>
+        <v>32.200000000000003</v>
       </c>
       <c r="AL6" s="22">
         <v>33.4</v>
       </c>
       <c r="AM6" s="23">
         <f t="shared" ref="AM6:AM48" si="2">IF(AK6&gt;0,$AK6-$AL6,"")</f>
-        <v>-1.8999999999999986</v>
+        <v>-1.1999999999999957</v>
       </c>
       <c r="AN6" s="23">
         <v>31.046424304488809</v>
@@ -9569,7 +9573,9 @@
       <c r="F7" s="63">
         <v>37.6</v>
       </c>
-      <c r="G7" s="63"/>
+      <c r="G7" s="63">
+        <v>36</v>
+      </c>
       <c r="H7" s="63"/>
       <c r="I7" s="63"/>
       <c r="J7" s="63"/>
@@ -9600,7 +9606,7 @@
       <c r="AI7" s="63"/>
       <c r="AJ7" s="36">
         <f t="shared" si="0"/>
-        <v>37.6</v>
+        <v>36</v>
       </c>
       <c r="AK7" s="21">
         <f t="shared" si="1"/>
@@ -9644,7 +9650,9 @@
       <c r="F8" s="63">
         <v>33</v>
       </c>
-      <c r="G8" s="63"/>
+      <c r="G8" s="63">
+        <v>34.4</v>
+      </c>
       <c r="H8" s="63"/>
       <c r="I8" s="63"/>
       <c r="J8" s="63"/>
@@ -9675,18 +9683,18 @@
       <c r="AI8" s="63"/>
       <c r="AJ8" s="36">
         <f t="shared" si="0"/>
-        <v>33</v>
+        <v>34.4</v>
       </c>
       <c r="AK8" s="21">
         <f t="shared" si="1"/>
-        <v>33.200000000000003</v>
+        <v>34.4</v>
       </c>
       <c r="AL8" s="22">
         <v>36.9</v>
       </c>
       <c r="AM8" s="23">
         <f t="shared" si="2"/>
-        <v>-3.6999999999999957</v>
+        <v>-2.5</v>
       </c>
       <c r="AN8" s="23">
         <v>32.243805889046577</v>
@@ -9719,7 +9727,9 @@
       <c r="F9" s="63">
         <v>36.299999999999997</v>
       </c>
-      <c r="G9" s="63"/>
+      <c r="G9" s="63">
+        <v>35.5</v>
+      </c>
       <c r="H9" s="63"/>
       <c r="I9" s="63"/>
       <c r="J9" s="63"/>
@@ -9750,7 +9760,7 @@
       <c r="AI9" s="63"/>
       <c r="AJ9" s="36">
         <f t="shared" si="0"/>
-        <v>36.299999999999997</v>
+        <v>35.5</v>
       </c>
       <c r="AK9" s="21">
         <f t="shared" si="1"/>
@@ -9794,7 +9804,9 @@
       <c r="F10" s="63">
         <v>37.9</v>
       </c>
-      <c r="G10" s="63"/>
+      <c r="G10" s="63">
+        <v>37.4</v>
+      </c>
       <c r="H10" s="63"/>
       <c r="I10" s="63"/>
       <c r="J10" s="63"/>
@@ -9825,7 +9837,7 @@
       <c r="AI10" s="63"/>
       <c r="AJ10" s="36">
         <f t="shared" si="0"/>
-        <v>37.9</v>
+        <v>37.4</v>
       </c>
       <c r="AK10" s="21">
         <f t="shared" si="1"/>
@@ -9869,7 +9881,9 @@
       <c r="F11" s="63">
         <v>40.6</v>
       </c>
-      <c r="G11" s="63"/>
+      <c r="G11" s="63">
+        <v>39.200000000000003</v>
+      </c>
       <c r="H11" s="63"/>
       <c r="I11" s="63"/>
       <c r="J11" s="63"/>
@@ -9900,7 +9914,7 @@
       <c r="AI11" s="63"/>
       <c r="AJ11" s="36">
         <f t="shared" si="0"/>
-        <v>40.6</v>
+        <v>39.200000000000003</v>
       </c>
       <c r="AK11" s="21">
         <f t="shared" si="1"/>
@@ -9944,7 +9958,9 @@
       <c r="F12" s="63">
         <v>35.799999999999997</v>
       </c>
-      <c r="G12" s="63"/>
+      <c r="G12" s="63">
+        <v>35.200000000000003</v>
+      </c>
       <c r="H12" s="63"/>
       <c r="I12" s="63"/>
       <c r="J12" s="63"/>
@@ -9975,7 +9991,7 @@
       <c r="AI12" s="63"/>
       <c r="AJ12" s="36">
         <f t="shared" si="0"/>
-        <v>35.799999999999997</v>
+        <v>35.200000000000003</v>
       </c>
       <c r="AK12" s="21">
         <f t="shared" si="1"/>
@@ -10019,7 +10035,9 @@
       <c r="F13" s="63">
         <v>36.799999999999997</v>
       </c>
-      <c r="G13" s="63"/>
+      <c r="G13" s="63">
+        <v>36.6</v>
+      </c>
       <c r="H13" s="63"/>
       <c r="I13" s="63"/>
       <c r="J13" s="63"/>
@@ -10050,7 +10068,7 @@
       <c r="AI13" s="63"/>
       <c r="AJ13" s="36">
         <f t="shared" si="0"/>
-        <v>36.799999999999997</v>
+        <v>36.6</v>
       </c>
       <c r="AK13" s="21">
         <f t="shared" si="1"/>
@@ -10094,7 +10112,9 @@
       <c r="F14" s="63">
         <v>35.700000000000003</v>
       </c>
-      <c r="G14" s="63"/>
+      <c r="G14" s="63">
+        <v>34.4</v>
+      </c>
       <c r="H14" s="63"/>
       <c r="I14" s="63"/>
       <c r="J14" s="63"/>
@@ -10125,7 +10145,7 @@
       <c r="AI14" s="63"/>
       <c r="AJ14" s="36">
         <f t="shared" si="0"/>
-        <v>35.700000000000003</v>
+        <v>34.4</v>
       </c>
       <c r="AK14" s="21">
         <f t="shared" si="1"/>
@@ -10169,7 +10189,9 @@
       <c r="F15" s="63">
         <v>32.9</v>
       </c>
-      <c r="G15" s="63"/>
+      <c r="G15" s="63">
+        <v>28.9</v>
+      </c>
       <c r="H15" s="63"/>
       <c r="I15" s="63"/>
       <c r="J15" s="63"/>
@@ -10200,7 +10222,7 @@
       <c r="AI15" s="63"/>
       <c r="AJ15" s="36">
         <f t="shared" si="0"/>
-        <v>32.9</v>
+        <v>28.9</v>
       </c>
       <c r="AK15" s="21">
         <f t="shared" si="1"/>
@@ -10293,7 +10315,9 @@
       <c r="F17" s="63">
         <v>36.200000000000003</v>
       </c>
-      <c r="G17" s="63"/>
+      <c r="G17" s="63">
+        <v>34.1</v>
+      </c>
       <c r="H17" s="63"/>
       <c r="I17" s="63"/>
       <c r="J17" s="63"/>
@@ -10324,7 +10348,7 @@
       <c r="AI17" s="63"/>
       <c r="AJ17" s="36">
         <f t="shared" si="0"/>
-        <v>36.200000000000003</v>
+        <v>34.1</v>
       </c>
       <c r="AK17" s="21">
         <f t="shared" si="1"/>
@@ -10368,7 +10392,9 @@
       <c r="F18" s="63">
         <v>30.5</v>
       </c>
-      <c r="G18" s="63"/>
+      <c r="G18" s="63">
+        <v>28.4</v>
+      </c>
       <c r="H18" s="63"/>
       <c r="I18" s="63"/>
       <c r="J18" s="63"/>
@@ -10399,7 +10425,7 @@
       <c r="AI18" s="63"/>
       <c r="AJ18" s="36">
         <f t="shared" si="0"/>
-        <v>30.5</v>
+        <v>28.4</v>
       </c>
       <c r="AK18" s="21">
         <f t="shared" si="1"/>
@@ -10443,7 +10469,9 @@
       <c r="F19" s="63">
         <v>36.1</v>
       </c>
-      <c r="G19" s="63"/>
+      <c r="G19" s="63">
+        <v>34.5</v>
+      </c>
       <c r="H19" s="63"/>
       <c r="I19" s="63"/>
       <c r="J19" s="63"/>
@@ -10474,7 +10502,7 @@
       <c r="AI19" s="63"/>
       <c r="AJ19" s="36">
         <f t="shared" si="0"/>
-        <v>36.1</v>
+        <v>34.5</v>
       </c>
       <c r="AK19" s="21">
         <f t="shared" si="1"/>
@@ -10518,7 +10546,9 @@
       <c r="F20" s="63">
         <v>30.9</v>
       </c>
-      <c r="G20" s="63"/>
+      <c r="G20" s="63">
+        <v>30</v>
+      </c>
       <c r="H20" s="63"/>
       <c r="I20" s="63"/>
       <c r="J20" s="63"/>
@@ -10549,7 +10579,7 @@
       <c r="AI20" s="63"/>
       <c r="AJ20" s="36">
         <f t="shared" si="0"/>
-        <v>30.9</v>
+        <v>30</v>
       </c>
       <c r="AK20" s="21">
         <f t="shared" si="1"/>
@@ -10593,7 +10623,9 @@
       <c r="F21" s="63">
         <v>24.5</v>
       </c>
-      <c r="G21" s="63"/>
+      <c r="G21" s="63">
+        <v>23.7</v>
+      </c>
       <c r="H21" s="63"/>
       <c r="I21" s="63"/>
       <c r="J21" s="63"/>
@@ -10624,7 +10656,7 @@
       <c r="AI21" s="63"/>
       <c r="AJ21" s="36">
         <f t="shared" si="0"/>
-        <v>24.5</v>
+        <v>23.7</v>
       </c>
       <c r="AK21" s="21">
         <f t="shared" si="1"/>
@@ -10736,7 +10768,9 @@
       <c r="F23" s="63">
         <v>31.4</v>
       </c>
-      <c r="G23" s="63"/>
+      <c r="G23" s="63">
+        <v>29</v>
+      </c>
       <c r="H23" s="63"/>
       <c r="I23" s="63"/>
       <c r="J23" s="63"/>
@@ -10767,7 +10801,7 @@
       <c r="AI23" s="63"/>
       <c r="AJ23" s="36">
         <f t="shared" si="0"/>
-        <v>31.4</v>
+        <v>29</v>
       </c>
       <c r="AK23" s="21">
         <f t="shared" si="1"/>
@@ -10811,7 +10845,9 @@
       <c r="F24" s="63">
         <v>32.200000000000003</v>
       </c>
-      <c r="G24" s="63"/>
+      <c r="G24" s="63">
+        <v>30.3</v>
+      </c>
       <c r="H24" s="63"/>
       <c r="I24" s="63"/>
       <c r="J24" s="63"/>
@@ -10842,7 +10878,7 @@
       <c r="AI24" s="63"/>
       <c r="AJ24" s="36">
         <f t="shared" si="0"/>
-        <v>32.200000000000003</v>
+        <v>30.3</v>
       </c>
       <c r="AK24" s="21">
         <f t="shared" si="1"/>
@@ -10886,7 +10922,9 @@
       <c r="F25" s="63">
         <v>36.1</v>
       </c>
-      <c r="G25" s="63"/>
+      <c r="G25" s="63">
+        <v>34.700000000000003</v>
+      </c>
       <c r="H25" s="63"/>
       <c r="I25" s="63"/>
       <c r="J25" s="63"/>
@@ -10917,7 +10955,7 @@
       <c r="AI25" s="63"/>
       <c r="AJ25" s="36">
         <f t="shared" si="0"/>
-        <v>36.1</v>
+        <v>34.700000000000003</v>
       </c>
       <c r="AK25" s="21">
         <f t="shared" si="1"/>
@@ -10961,7 +10999,9 @@
       <c r="F26" s="63">
         <v>20.5</v>
       </c>
-      <c r="G26" s="63"/>
+      <c r="G26" s="63">
+        <v>19.3</v>
+      </c>
       <c r="H26" s="63"/>
       <c r="I26" s="63"/>
       <c r="J26" s="63"/>
@@ -10992,7 +11032,7 @@
       <c r="AI26" s="63"/>
       <c r="AJ26" s="36">
         <f t="shared" si="0"/>
-        <v>20.5</v>
+        <v>19.3</v>
       </c>
       <c r="AK26" s="21">
         <f t="shared" si="1"/>
@@ -11036,7 +11076,9 @@
       <c r="F27" s="63">
         <v>20.399999999999999</v>
       </c>
-      <c r="G27" s="63"/>
+      <c r="G27" s="63">
+        <v>20.8</v>
+      </c>
       <c r="H27" s="63"/>
       <c r="I27" s="63"/>
       <c r="J27" s="63"/>
@@ -11067,18 +11109,18 @@
       <c r="AI27" s="63"/>
       <c r="AJ27" s="36">
         <f t="shared" si="0"/>
-        <v>20.399999999999999</v>
+        <v>20.8</v>
       </c>
       <c r="AK27" s="21">
         <f t="shared" si="1"/>
-        <v>20.399999999999999</v>
+        <v>20.8</v>
       </c>
       <c r="AL27" s="22">
         <v>22.4</v>
       </c>
       <c r="AM27" s="23">
         <f t="shared" si="2"/>
-        <v>-2</v>
+        <v>-1.5999999999999979</v>
       </c>
       <c r="AN27" s="23">
         <v>17.087318670151451</v>
@@ -11111,7 +11153,9 @@
       <c r="F28" s="63">
         <v>34.299999999999997</v>
       </c>
-      <c r="G28" s="63"/>
+      <c r="G28" s="63">
+        <v>30.1</v>
+      </c>
       <c r="H28" s="63"/>
       <c r="I28" s="63"/>
       <c r="J28" s="63"/>
@@ -11142,7 +11186,7 @@
       <c r="AI28" s="63"/>
       <c r="AJ28" s="36">
         <f t="shared" si="0"/>
-        <v>34.299999999999997</v>
+        <v>30.1</v>
       </c>
       <c r="AK28" s="21">
         <f t="shared" si="1"/>
@@ -11252,7 +11296,9 @@
       <c r="F30" s="63">
         <v>38.200000000000003</v>
       </c>
-      <c r="G30" s="63"/>
+      <c r="G30" s="63">
+        <v>36</v>
+      </c>
       <c r="H30" s="63"/>
       <c r="I30" s="63"/>
       <c r="J30" s="63"/>
@@ -11283,7 +11329,7 @@
       <c r="AI30" s="63"/>
       <c r="AJ30" s="36">
         <f t="shared" si="0"/>
-        <v>38.200000000000003</v>
+        <v>36</v>
       </c>
       <c r="AK30" s="21">
         <f t="shared" si="1"/>
@@ -11327,7 +11373,9 @@
       <c r="F31" s="63">
         <v>27.5</v>
       </c>
-      <c r="G31" s="63"/>
+      <c r="G31" s="63">
+        <v>27.2</v>
+      </c>
       <c r="H31" s="63"/>
       <c r="I31" s="63"/>
       <c r="J31" s="63"/>
@@ -11358,7 +11406,7 @@
       <c r="AI31" s="63"/>
       <c r="AJ31" s="36">
         <f t="shared" si="0"/>
-        <v>27.5</v>
+        <v>27.2</v>
       </c>
       <c r="AK31" s="21">
         <f t="shared" si="1"/>
@@ -11402,7 +11450,9 @@
       <c r="F32" s="63">
         <v>19</v>
       </c>
-      <c r="G32" s="63"/>
+      <c r="G32" s="63">
+        <v>15.6</v>
+      </c>
       <c r="H32" s="63"/>
       <c r="I32" s="63"/>
       <c r="J32" s="63"/>
@@ -11433,7 +11483,7 @@
       <c r="AI32" s="63"/>
       <c r="AJ32" s="36">
         <f t="shared" si="0"/>
-        <v>19</v>
+        <v>15.6</v>
       </c>
       <c r="AK32" s="21">
         <f t="shared" si="1"/>
@@ -11477,7 +11527,9 @@
       <c r="F33" s="63">
         <v>16</v>
       </c>
-      <c r="G33" s="63"/>
+      <c r="G33" s="63">
+        <v>14.8</v>
+      </c>
       <c r="H33" s="63"/>
       <c r="I33" s="63"/>
       <c r="J33" s="63"/>
@@ -11508,7 +11560,7 @@
       <c r="AI33" s="63"/>
       <c r="AJ33" s="36">
         <f t="shared" si="0"/>
-        <v>16</v>
+        <v>14.8</v>
       </c>
       <c r="AK33" s="21">
         <f t="shared" si="1"/>
@@ -11604,7 +11656,9 @@
       <c r="F35" s="63">
         <v>34.799999999999997</v>
       </c>
-      <c r="G35" s="63"/>
+      <c r="G35" s="63">
+        <v>30</v>
+      </c>
       <c r="H35" s="63"/>
       <c r="I35" s="63"/>
       <c r="J35" s="63"/>
@@ -11635,7 +11689,7 @@
       <c r="AI35" s="63"/>
       <c r="AJ35" s="36">
         <f t="shared" si="0"/>
-        <v>34.799999999999997</v>
+        <v>30</v>
       </c>
       <c r="AK35" s="21">
         <f t="shared" si="1"/>
@@ -11800,7 +11854,9 @@
       <c r="F38" s="63">
         <v>34.1</v>
       </c>
-      <c r="G38" s="63"/>
+      <c r="G38" s="63">
+        <v>32.5</v>
+      </c>
       <c r="H38" s="63"/>
       <c r="I38" s="63"/>
       <c r="J38" s="63"/>
@@ -11831,7 +11887,7 @@
       <c r="AI38" s="63"/>
       <c r="AJ38" s="36">
         <f t="shared" si="0"/>
-        <v>34.1</v>
+        <v>32.5</v>
       </c>
       <c r="AK38" s="21">
         <f t="shared" si="1"/>
@@ -11876,7 +11932,9 @@
       <c r="F39" s="63">
         <v>32</v>
       </c>
-      <c r="G39" s="63"/>
+      <c r="G39" s="63">
+        <v>32.4</v>
+      </c>
       <c r="H39" s="63"/>
       <c r="I39" s="63"/>
       <c r="J39" s="63"/>
@@ -11907,7 +11965,7 @@
       <c r="AI39" s="63"/>
       <c r="AJ39" s="36">
         <f t="shared" si="0"/>
-        <v>32</v>
+        <v>32.4</v>
       </c>
       <c r="AK39" s="21">
         <f t="shared" si="1"/>
@@ -11952,7 +12010,9 @@
       <c r="F40" s="63">
         <v>32</v>
       </c>
-      <c r="G40" s="63"/>
+      <c r="G40" s="63">
+        <v>30.6</v>
+      </c>
       <c r="H40" s="63"/>
       <c r="I40" s="63"/>
       <c r="J40" s="63"/>
@@ -11983,7 +12043,7 @@
       <c r="AI40" s="63"/>
       <c r="AJ40" s="36">
         <f t="shared" si="0"/>
-        <v>32</v>
+        <v>30.6</v>
       </c>
       <c r="AK40" s="21">
         <f t="shared" si="1"/>
@@ -12028,7 +12088,9 @@
       <c r="F41" s="63">
         <v>33.6</v>
       </c>
-      <c r="G41" s="63"/>
+      <c r="G41" s="63">
+        <v>31.6</v>
+      </c>
       <c r="H41" s="63"/>
       <c r="I41" s="63"/>
       <c r="J41" s="63"/>
@@ -12059,7 +12121,7 @@
       <c r="AI41" s="63"/>
       <c r="AJ41" s="36">
         <f t="shared" si="0"/>
-        <v>33.6</v>
+        <v>31.6</v>
       </c>
       <c r="AK41" s="21">
         <f t="shared" si="1"/>
@@ -12171,7 +12233,9 @@
       <c r="F43" s="63">
         <v>31.8</v>
       </c>
-      <c r="G43" s="63"/>
+      <c r="G43" s="63">
+        <v>32.200000000000003</v>
+      </c>
       <c r="H43" s="63"/>
       <c r="I43" s="63"/>
       <c r="J43" s="63"/>
@@ -12202,18 +12266,18 @@
       <c r="AI43" s="63"/>
       <c r="AJ43" s="36">
         <f t="shared" si="0"/>
-        <v>31.8</v>
+        <v>32.200000000000003</v>
       </c>
       <c r="AK43" s="21">
         <f t="shared" si="1"/>
-        <v>32</v>
+        <v>32.200000000000003</v>
       </c>
       <c r="AL43" s="22">
         <v>35.4</v>
       </c>
       <c r="AM43" s="23">
         <f t="shared" si="2"/>
-        <v>-3.3999999999999986</v>
+        <v>-3.1999999999999957</v>
       </c>
       <c r="AN43" s="23">
         <v>31.022074370307589</v>
@@ -12247,7 +12311,9 @@
       <c r="F44" s="29">
         <v>31</v>
       </c>
-      <c r="G44" s="29"/>
+      <c r="G44" s="29">
+        <v>31.3</v>
+      </c>
       <c r="H44" s="29"/>
       <c r="I44" s="29"/>
       <c r="J44" s="29"/>
@@ -12278,7 +12344,7 @@
       <c r="AI44" s="63"/>
       <c r="AJ44" s="36">
         <f t="shared" si="0"/>
-        <v>31</v>
+        <v>31.3</v>
       </c>
       <c r="AK44" s="21">
         <f t="shared" si="1"/>
@@ -12323,7 +12389,9 @@
       <c r="F45" s="63">
         <v>33.200000000000003</v>
       </c>
-      <c r="G45" s="63"/>
+      <c r="G45" s="63">
+        <v>32</v>
+      </c>
       <c r="H45" s="63"/>
       <c r="I45" s="63"/>
       <c r="J45" s="63"/>
@@ -12354,7 +12422,7 @@
       <c r="AI45" s="63"/>
       <c r="AJ45" s="36">
         <f t="shared" si="0"/>
-        <v>33.200000000000003</v>
+        <v>32</v>
       </c>
       <c r="AK45" s="21">
         <f t="shared" si="1"/>
@@ -12538,7 +12606,9 @@
       <c r="F48" s="63">
         <v>32.6</v>
       </c>
-      <c r="G48" s="63"/>
+      <c r="G48" s="63">
+        <v>31.9</v>
+      </c>
       <c r="H48" s="63"/>
       <c r="I48" s="63"/>
       <c r="J48" s="63"/>
@@ -12569,7 +12639,7 @@
       <c r="AI48" s="63"/>
       <c r="AJ48" s="36">
         <f t="shared" si="0"/>
-        <v>32.6</v>
+        <v>31.9</v>
       </c>
       <c r="AK48" s="21">
         <f t="shared" si="1"/>
@@ -25492,12 +25562,6 @@
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:D2"/>
-    <mergeCell ref="E1:E2"/>
     <mergeCell ref="M1:M2"/>
     <mergeCell ref="N1:N2"/>
     <mergeCell ref="O1:O2"/>
@@ -25507,6 +25571,12 @@
     <mergeCell ref="J1:J2"/>
     <mergeCell ref="K1:K2"/>
     <mergeCell ref="L1:L2"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="E1:E2"/>
   </mergeCells>
   <conditionalFormatting sqref="D4:O13 D15:O31 D33:O34 D36:O46">
     <cfRule type="cellIs" dxfId="0" priority="1" stopIfTrue="1" operator="equal">

</xml_diff>